<commit_message>
Slack Integration - Complete
</commit_message>
<xml_diff>
--- a/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
+++ b/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
@@ -2,9 +2,6 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
-  <bookViews>
-    <workbookView activeTab="0"/>
-  </bookViews>
   <sheets>
     <sheet state="visible" name="test_suite" sheetId="1" r:id="rId4"/>
     <sheet state="visible" name="validData" sheetId="2" r:id="rId5"/>
@@ -22,12 +19,13 @@
     <sheet state="visible" name="overAllAcademicsTest" sheetId="14" r:id="rId17"/>
     <sheet state="visible" name="CollegeUniversitiesTest" sheetId="15" r:id="rId18"/>
   </sheets>
+  <definedNames/>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="102">
   <si>
     <t>TCID</t>
   </si>
@@ -333,25 +331,12 @@
   </si>
   <si>
     <t>Test Degree</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>112419@test.asu.edu</t>
-  </si>
-  <si>
-    <t>Date of birth</t>
-  </si>
-  <si>
-    <t>May 24, 1988</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="0"/>
   <fonts count="10">
     <font>
       <sz val="11.0"/>
@@ -432,7 +417,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -455,12 +440,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf quotePrefix="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -728,11 +707,10 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1000"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="24.57"/>
-    <col min="2" max="6" customWidth="true" width="8.71"/>
+    <col customWidth="1" min="1" max="1" width="24.57"/>
+    <col customWidth="1" min="2" max="6" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2449,15 +2427,14 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="38.29"/>
-    <col min="3" max="3" customWidth="true" width="34.0"/>
-    <col min="4" max="4" customWidth="true" width="22.29"/>
-    <col min="5" max="5" customWidth="true" width="30.0"/>
-    <col min="6" max="6" customWidth="true" width="18.57"/>
-    <col min="7" max="7" customWidth="true" width="30.14"/>
+    <col customWidth="1" min="1" max="2" width="38.29"/>
+    <col customWidth="1" min="3" max="3" width="34.0"/>
+    <col customWidth="1" min="4" max="4" width="22.29"/>
+    <col customWidth="1" min="5" max="5" width="30.0"/>
+    <col customWidth="1" min="6" max="6" width="18.57"/>
+    <col customWidth="1" min="7" max="7" width="30.14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2552,14 +2529,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="38.29"/>
-    <col min="3" max="3" customWidth="true" width="34.0"/>
-    <col min="4" max="4" customWidth="true" width="22.29"/>
-    <col min="5" max="5" customWidth="true" width="30.0"/>
-    <col min="6" max="6" customWidth="true" width="14.43"/>
+    <col customWidth="1" min="1" max="2" width="38.29"/>
+    <col customWidth="1" min="3" max="3" width="34.0"/>
+    <col customWidth="1" min="4" max="4" width="22.29"/>
+    <col customWidth="1" min="5" max="5" width="30.0"/>
+    <col customWidth="1" min="6" max="6" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2636,14 +2612,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.14"/>
-    <col min="2" max="2" customWidth="true" width="29.57"/>
-    <col min="3" max="3" customWidth="true" width="41.43"/>
-    <col min="4" max="4" customWidth="true" width="34.43"/>
-    <col min="5" max="5" customWidth="true" width="14.43"/>
+    <col customWidth="1" min="1" max="1" width="27.14"/>
+    <col customWidth="1" min="2" max="2" width="29.57"/>
+    <col customWidth="1" min="3" max="3" width="41.43"/>
+    <col customWidth="1" min="4" max="4" width="34.43"/>
+    <col customWidth="1" min="5" max="5" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2711,10 +2686,9 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="5" customWidth="true" width="14.43"/>
+    <col customWidth="1" min="1" max="5" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2901,10 +2875,9 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="4" customWidth="true" width="14.43"/>
+    <col customWidth="1" min="1" max="4" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3001,14 +2974,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="31.0"/>
-    <col min="2" max="2" customWidth="true" width="27.43"/>
-    <col min="3" max="3" customWidth="true" width="51.0"/>
-    <col min="4" max="4" customWidth="true" width="22.43"/>
-    <col min="5" max="5" customWidth="true" width="14.43"/>
+    <col customWidth="1" min="1" max="1" width="31.0"/>
+    <col customWidth="1" min="2" max="2" width="27.43"/>
+    <col customWidth="1" min="3" max="3" width="51.0"/>
+    <col customWidth="1" min="4" max="4" width="22.43"/>
+    <col customWidth="1" min="5" max="5" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3075,26 +3047,20 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="36.86"/>
-    <col min="2" max="2" customWidth="true" width="41.14"/>
-    <col min="3" max="3" customWidth="true" width="20.43"/>
-    <col min="4" max="4" customWidth="true" width="20.14"/>
-    <col min="5" max="5" customWidth="true" width="31.43"/>
-    <col min="6" max="6" customWidth="true" width="24.43"/>
-    <col min="7" max="7" customWidth="true" width="26.71"/>
-    <col min="12" max="12" customWidth="true" width="40.71"/>
+    <col customWidth="1" min="1" max="1" width="36.86"/>
+    <col customWidth="1" min="2" max="2" width="41.14"/>
+    <col customWidth="1" min="3" max="3" width="20.43"/>
+    <col customWidth="1" min="4" max="4" width="20.14"/>
+    <col customWidth="1" min="5" max="5" width="31.43"/>
+    <col customWidth="1" min="6" max="6" width="24.43"/>
+    <col customWidth="1" min="7" max="7" width="26.71"/>
+    <col customWidth="1" min="12" max="12" width="40.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" t="s" s="0">
-        <v>102</v>
-      </c>
-      <c r="B1" s="14" t="s">
-        <v>103</v>
-      </c>
+      <c r="B1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="4"/>
       <c r="F1" s="3"/>
@@ -3124,12 +3090,8 @@
       <c r="L3" s="3"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" t="s" s="0">
-        <v>104</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>105</v>
-      </c>
+      <c r="A4" s="4"/>
+      <c r="B4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="4"/>
       <c r="F4" s="3"/>
@@ -5236,15 +5198,14 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="13.14"/>
-    <col min="2" max="2" customWidth="true" width="23.71"/>
-    <col min="3" max="3" customWidth="true" width="45.14"/>
-    <col min="4" max="4" customWidth="true" width="14.57"/>
-    <col min="5" max="5" customWidth="true" width="60.0"/>
-    <col min="6" max="6" customWidth="true" width="25.14"/>
+    <col customWidth="1" min="1" max="1" width="13.14"/>
+    <col customWidth="1" min="2" max="2" width="23.71"/>
+    <col customWidth="1" min="3" max="3" width="45.14"/>
+    <col customWidth="1" min="4" max="4" width="14.57"/>
+    <col customWidth="1" min="5" max="5" width="60.0"/>
+    <col customWidth="1" min="6" max="6" width="25.14"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -7307,15 +7268,14 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="37.29"/>
-    <col min="2" max="2" customWidth="true" width="29.57"/>
-    <col min="3" max="3" customWidth="true" width="24.57"/>
-    <col min="4" max="4" customWidth="true" width="27.57"/>
-    <col min="5" max="5" customWidth="true" width="25.29"/>
-    <col min="6" max="6" customWidth="true" width="33.57"/>
+    <col customWidth="1" min="1" max="1" width="37.29"/>
+    <col customWidth="1" min="2" max="2" width="29.57"/>
+    <col customWidth="1" min="3" max="3" width="24.57"/>
+    <col customWidth="1" min="4" max="4" width="27.57"/>
+    <col customWidth="1" min="5" max="5" width="25.29"/>
+    <col customWidth="1" min="6" max="6" width="33.57"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9374,12 +9334,11 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.29"/>
-    <col min="2" max="2" customWidth="true" width="14.14"/>
-    <col min="3" max="3" customWidth="true" width="8.71"/>
+    <col customWidth="1" min="1" max="1" width="27.29"/>
+    <col customWidth="1" min="2" max="2" width="14.14"/>
+    <col customWidth="1" min="3" max="3" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9442,14 +9401,13 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="29.43"/>
-    <col min="2" max="2" customWidth="true" width="31.43"/>
-    <col min="3" max="3" customWidth="true" width="28.71"/>
-    <col min="4" max="4" customWidth="true" width="30.57"/>
-    <col min="5" max="5" customWidth="true" width="8.71"/>
+    <col customWidth="1" min="1" max="1" width="29.43"/>
+    <col customWidth="1" min="2" max="2" width="31.43"/>
+    <col customWidth="1" min="3" max="3" width="28.71"/>
+    <col customWidth="1" min="4" max="4" width="30.57"/>
+    <col customWidth="1" min="5" max="5" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9567,13 +9525,12 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.29"/>
-    <col min="2" max="2" customWidth="true" width="20.14"/>
-    <col min="3" max="4" customWidth="true" width="13.57"/>
-    <col min="5" max="5" customWidth="true" width="8.71"/>
+    <col customWidth="1" min="1" max="1" width="27.29"/>
+    <col customWidth="1" min="2" max="2" width="20.14"/>
+    <col customWidth="1" min="3" max="4" width="13.57"/>
+    <col customWidth="1" min="5" max="5" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9675,12 +9632,11 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.57"/>
-    <col min="2" max="2" customWidth="true" width="39.86"/>
-    <col min="3" max="3" customWidth="true" width="14.43"/>
+    <col customWidth="1" min="1" max="1" width="27.57"/>
+    <col customWidth="1" min="2" max="2" width="39.86"/>
+    <col customWidth="1" min="3" max="3" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9862,12 +9818,11 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="56.0"/>
-    <col min="2" max="2" customWidth="true" width="57.0"/>
-    <col min="3" max="3" customWidth="true" width="14.43"/>
+    <col customWidth="1" min="1" max="1" width="56.0"/>
+    <col customWidth="1" min="2" max="2" width="57.0"/>
+    <col customWidth="1" min="3" max="3" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
3/2/25 - Create account, LogIn, Email verification pages Xpaths updates
</commit_message>
<xml_diff>
--- a/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
+++ b/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
@@ -25,14 +25,13 @@
     <sheet name="AddMaxHighSchoolTest" sheetId="13" r:id="rId13"/>
     <sheet name="overAllAcademicsTest" sheetId="14" r:id="rId14"/>
     <sheet name="CollegeUniversitiesTest" sheetId="15" r:id="rId15"/>
-    <sheet name="Mismatch_01_valid_vs_Revie" r:id="rId19" sheetId="16"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>TCID</t>
   </si>
@@ -343,12 +342,6 @@
     <t>Test Degree</t>
   </si>
   <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>5382521@test.asu.edu</t>
-  </si>
-  <si>
     <t>Legal name</t>
   </si>
   <si>
@@ -358,435 +351,10 @@
     <t>Preferred first name</t>
   </si>
   <si>
-    <t>Legal sex</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>Primary language spoken at home</t>
-  </si>
-  <si>
-    <t>Chhattisgarhi</t>
-  </si>
-  <si>
-    <t>Home address</t>
-  </si>
-  <si>
-    <t>Test Address Line I Test Address Line II
-Test City,Arizona,United States
-United States
-Afghanistan
-Aland Islands
-Albania
-Algeria
-American Samoa
-Andorra
-Angola
-Anguilla
-Antarctica
-Antigua and Barbuda
-Argentina
-Armenia
-Aruba
-Australia
-Austria
-Azerbaijan
-Bahamas, The
-Bahrain
-Bangladesh
-Barbados
-Belarus
-Belgium
-Belize
-Benin
-Bermuda
-Bhutan
-Bolivia
-Bonaire, Sint Eustatius &amp; Saba
-Bosnia and Herzegovina
-Botswana
-Bouvet Island
-Brazil
-British Indian Ocean Territory
-British Virgin Islands
-Brunei
-Bulgaria
-Burkina Faso
-Burma
-Burundi
-Cambodia
-Cameroon
-Canada
-Cape Verde
-Cayman Islands
-Central African Republic
-Chad
-Chile
-China
-Christmas Island
-Cocos (Keeling) Islands
-Colombia
-Comoros
-Congo
-Congo, Democratic Republic of
-Cook Islands
-Costa Rica
-Cote D'Ivoire
-Croatia
-Cuba
-Curacao
-Cyprus
-Czech Republic
-Denmark
-Djibouti
-Dominica
-Dominican Republic
-Ecuador
-Egypt
-El Salvador
-Equatorial Guinea
-Eritrea
-Estonia
-Eswatini
-Ethiopia
-Falkland Islands (Malvinas)
-Faroe Islands
-Fiji
-Finland
-France
-French Guiana
-French Polynesia
-French Southern &amp; Antarc Lands
-Gabon
-Gambia, The
-Georgia
-Germany
-Ghana
-Gibraltar
-Greece
-Greenland
-Grenada
-Guadeloupe
-Guam
-Guatemala
-Guernsey
-Guinea
-Guinea-Bissau
-Guyana
-Haiti
-Heard and McDonald Islands
-Honduras
-Hong Kong
-Hungary
-Iceland
-India
-Indonesia
-Iran
-Iraq
-Ireland
-Isle of Man
-Israel
-Italy
-Jamaica
-Japan
-Jersey
-Jordan
-Kazakhstan
-Kenya
-Kiribati
-Kosovo
-Kuwait
-Kyrgyzstan
-Laos
-Latvia
-Lebanon
-Lesotho
-Liberia
-Libya
-Liechtenstein
-Lithuania
-Luxembourg
-Macau
-Madagascar
-Malawi
-Malaysia
-Maldives
-Mali
-Malta
-Marshall Islands
-Martinique
-Mauritania
-Mauritius
-Mayotte
-Mexico
-Micronesia, Federated States
-Moldova
-Monaco
-Mongolia
-Montenegro
-Montserrat
-Morocco
-Mozambique
-Namibia
-Nauru
-Nepal
-Netherlands
-Netherlands Antilles
-New Caledonia
-New Zealand
-Nicaragua
-Niger
-Nigeria
-Niue
-Norfolk Island
-North Korea
-Northern Mariana Islands
-Norway
-Oman
-Pakistan
-Palau
-Palestinian Territory, Occupie
-Panama
-Papua New Guinea
-Paraguay
-Peru
-Philippines
-Pitcairn Islands
-Poland
-Portugal
-Puerto Rico
-Qatar
-Republic of North Macedonia
-Reunion
-Romania
-Russia
-Rwanda
-Saint Barthelemy
-Saint Helena
-Saint Kitts and Nevis
-Saint Lucia
-Saint Martin
-Saint Pierre and Miquelon
-Saint Vincent &amp; the Grenadines
-Samoa
-San Marino
-Sao Tome and Principe
-Saudi Arabia
-Senegal
-Serbia
-Seychelles
-Sierra Leone
-Singapore
-Sint Maarten (Dutch part)
-Slovakia
-Slovenia
-Solomon Islands
-Somalia
-South Africa
-South Georgia &amp; S Sandwich Is
-South Korea
-South Sudan
-Spain
-Spratly Islands
-Sri Lanka
-Sudan
-Suriname
-Svalbard and Jan Mayen
-Sweden
-Switzerland
-Syria
-Taiwan
-Tajikistan
-Tanzania
-Thailand
-Timor-Leste
-Togo
-Tokelau
-Tonga
-Trinidad and Tobago
-Tunisia
-Turkey
-Turkmenistan
-Turks and Caicos Islands
-Tuvalu
-US Misc Pacific Islands
-Uganda
-Ukraine
-United Arab Emirates
-United Kingdom
-Uruguay
-Uzbekistan
-Vanuatu
-Vatican City
-Venezuela
-Vietnam
-Virgin Islands
-Wallis and Futuna Islands
-Western Sahara
-Yemen
-Yugoslavia
-Zambia
-Zimbabwe
-12345-678910</t>
-  </si>
-  <si>
-    <t>U.S. citizenship</t>
-  </si>
-  <si>
-    <t>I am a U.S. citizen</t>
-  </si>
-  <si>
-    <t>Country of citizenship</t>
-  </si>
-  <si>
-    <t>United States</t>
-  </si>
-  <si>
-    <t>Country of birth</t>
-  </si>
-  <si>
-    <t>South Korea</t>
-  </si>
-  <si>
-    <t>Social Security Number</t>
-  </si>
-  <si>
-    <t>*********</t>
-  </si>
-  <si>
-    <t>Previous ASU affiliation</t>
-  </si>
-  <si>
-    <t>I have never been affiliated with Arizona State University</t>
-  </si>
-  <si>
-    <t>Military status</t>
-  </si>
-  <si>
-    <t>None of these options apply to me</t>
-  </si>
-  <si>
-    <t>Do you plan to use an education benefit or scholarship through an employer, corporation, foundation or other ASU education partner?</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Graduating school </t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>High school name</t>
-  </si>
-  <si>
-    <t>Name on transcript</t>
-  </si>
-  <si>
-    <t>Test FN Test LN</t>
-  </si>
-  <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>Test City, BS, GNQ</t>
-  </si>
-  <si>
-    <t>Graduation date</t>
-  </si>
-  <si>
-    <t>July, 2027</t>
-  </si>
-  <si>
-    <t>Transfer credits to ASU</t>
-  </si>
-  <si>
-    <t>Begin by selecting the state you consider to be your permanent home.</t>
-  </si>
-  <si>
-    <t>Outside the U.S. or Not Listed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In which state do your parent(s) or legal guardian(s) currently live? </t>
-  </si>
-  <si>
-    <t>New Hampshire</t>
-  </si>
-  <si>
     <t>Date of birth</t>
   </si>
   <si>
-    <t>November 11, 2010</t>
-  </si>
-  <si>
-    <t>Pronouns</t>
-  </si>
-  <si>
-    <t>No data has been entered</t>
-  </si>
-  <si>
-    <t>Gender identity</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>+1 (234) 567-6543</t>
-  </si>
-  <si>
-    <t>Mobile phone</t>
-  </si>
-  <si>
-    <t>Mobile SMS</t>
-  </si>
-  <si>
-    <t>Former name(s)</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Test Address Line I Test Address Line II
-Test City,Arizona,United States
-12345-678910</t>
-  </si>
-  <si>
-    <t>Ethnic/racial background</t>
-  </si>
-  <si>
-    <t>Affiliate ID</t>
-  </si>
-  <si>
-    <t>Program</t>
-  </si>
-  <si>
-    <t>Nondegree</t>
-  </si>
-  <si>
-    <t>ASU Online</t>
-  </si>
-  <si>
-    <t>Starting term</t>
-  </si>
-  <si>
-    <t>Fall 2025 - (Session B)</t>
-  </si>
-  <si>
-    <t>Graduating school</t>
-  </si>
-  <si>
-    <t>Key</t>
-  </si>
-  <si>
-    <t>Value Sheet 1</t>
-  </si>
-  <si>
-    <t>Value Sheet 2</t>
-  </si>
-  <si>
-    <t>In which state do your parent(s) or legal guardian(s) currently live?</t>
+    <t>November 13, 1964</t>
   </si>
 </sst>
 </file>
@@ -865,7 +433,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -888,252 +456,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment wrapText="true"/>
     </xf>
@@ -3673,38 +2995,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
-        <v>162</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>163</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>112</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>113</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>153</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:L1000"/>
@@ -3721,12 +3011,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" t="s" s="0">
-        <v>103</v>
-      </c>
-      <c r="B1" s="14" t="s">
-        <v>104</v>
-      </c>
+      <c r="B1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="1"/>
       <c r="F1" s="3"/>
@@ -3737,10 +3022,10 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" t="s" s="0">
-        <v>105</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>106</v>
+        <v>103</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>104</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="1"/>
@@ -3751,9 +3036,9 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" t="s" s="0">
-        <v>107</v>
-      </c>
-      <c r="B3" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>29</v>
       </c>
       <c r="D3" s="3"/>
@@ -3764,8 +3049,12 @@
       <c r="L3" s="3"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" s="1"/>
-      <c r="B4" s="3"/>
+      <c r="A4" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>107</v>
+      </c>
       <c r="D4" s="3"/>
       <c r="E4" s="1"/>
       <c r="F4" s="3"/>
@@ -3803,12 +3092,7 @@
       <c r="H7" s="3"/>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="A8" t="s" s="0">
-        <v>108</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>109</v>
-      </c>
+      <c r="B8" s="4"/>
       <c r="D8" s="3"/>
       <c r="E8" s="1"/>
       <c r="F8" s="3"/>
@@ -3817,12 +3101,7 @@
       <c r="L8" s="3"/>
     </row>
     <row r="9" ht="14.25" customHeight="1">
-      <c r="A9" t="s" s="0">
-        <v>110</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>111</v>
-      </c>
+      <c r="B9" s="4"/>
       <c r="D9" s="3"/>
       <c r="E9" s="1"/>
       <c r="F9" s="3"/>
@@ -3831,12 +3110,7 @@
       <c r="L9" s="3"/>
     </row>
     <row r="10" ht="137.25" customHeight="1">
-      <c r="A10" t="s" s="0">
-        <v>112</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>113</v>
-      </c>
+      <c r="B10" s="4"/>
       <c r="D10" s="3"/>
       <c r="E10" s="1"/>
       <c r="F10" s="3"/>
@@ -3878,12 +3152,8 @@
       <c r="L13" s="3"/>
     </row>
     <row r="14" ht="14.25" customHeight="1">
-      <c r="A14" t="s" s="0">
-        <v>114</v>
-      </c>
-      <c r="B14" s="20" t="s">
-        <v>115</v>
-      </c>
+      <c r="A14" s="1"/>
+      <c r="B14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="1"/>
       <c r="F14" s="3"/>
@@ -3892,12 +3162,8 @@
       <c r="L14" s="3"/>
     </row>
     <row r="15" ht="14.25" customHeight="1">
-      <c r="A15" t="s" s="0">
-        <v>116</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>117</v>
-      </c>
+      <c r="A15" s="1"/>
+      <c r="B15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="1"/>
       <c r="F15" s="3"/>
@@ -3906,12 +3172,8 @@
       <c r="L15" s="3"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="A16" t="s" s="0">
-        <v>118</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>119</v>
-      </c>
+      <c r="A16" s="1"/>
+      <c r="B16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="1"/>
       <c r="F16" s="3"/>
@@ -3920,12 +3182,8 @@
       <c r="L16" s="3"/>
     </row>
     <row r="17" ht="14.25" customHeight="1">
-      <c r="A17" t="s" s="0">
-        <v>120</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>121</v>
-      </c>
+      <c r="A17" s="1"/>
+      <c r="B17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="1"/>
       <c r="F17" s="3"/>
@@ -3981,12 +3239,8 @@
       <c r="B26" s="3"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
-      <c r="A27" t="s" s="0">
-        <v>122</v>
-      </c>
-      <c r="B27" s="24" t="s">
-        <v>123</v>
-      </c>
+      <c r="A27" s="1"/>
+      <c r="B27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="1"/>
       <c r="F27" s="3"/>
@@ -4005,12 +3259,8 @@
       <c r="L28" s="3"/>
     </row>
     <row r="29" ht="14.25" customHeight="1">
-      <c r="A29" t="s" s="0">
-        <v>124</v>
-      </c>
-      <c r="B29" s="25" t="s">
-        <v>125</v>
-      </c>
+      <c r="A29" s="1"/>
+      <c r="B29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="1"/>
       <c r="F29" s="3"/>
@@ -4046,12 +3296,8 @@
       <c r="L32" s="3"/>
     </row>
     <row r="33" ht="14.25" customHeight="1">
-      <c r="A33" t="s" s="0">
-        <v>126</v>
-      </c>
-      <c r="B33" s="26" t="s">
-        <v>127</v>
-      </c>
+      <c r="A33" s="1"/>
+      <c r="B33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="1"/>
       <c r="F33" s="3"/>
@@ -4179,12 +3425,8 @@
       <c r="L44" s="3"/>
     </row>
     <row r="45" ht="14.25" customHeight="1">
-      <c r="A45" t="s" s="0">
-        <v>128</v>
-      </c>
-      <c r="B45" s="27" t="s">
-        <v>129</v>
-      </c>
+      <c r="A45" s="1"/>
+      <c r="B45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="1"/>
       <c r="F45" s="3"/>
@@ -4195,12 +3437,8 @@
       <c r="L45" s="3"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
-      <c r="A46" t="s" s="0">
-        <v>130</v>
-      </c>
-      <c r="B46" s="28" t="s">
-        <v>79</v>
-      </c>
+      <c r="A46" s="1"/>
+      <c r="B46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="1"/>
       <c r="F46" s="3"/>
@@ -4211,12 +3449,8 @@
       <c r="L46" s="3"/>
     </row>
     <row r="47" ht="14.25" customHeight="1">
-      <c r="A47" t="s" s="0">
-        <v>131</v>
-      </c>
-      <c r="B47" s="29" t="s">
-        <v>132</v>
-      </c>
+      <c r="A47" s="1"/>
+      <c r="B47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="1"/>
       <c r="F47" s="3"/>
@@ -4227,12 +3461,8 @@
       <c r="L47" s="3"/>
     </row>
     <row r="48" ht="14.25" customHeight="1">
-      <c r="A48" t="s" s="0">
-        <v>133</v>
-      </c>
-      <c r="B48" s="30" t="s">
-        <v>134</v>
-      </c>
+      <c r="A48" s="1"/>
+      <c r="B48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="1"/>
       <c r="F48" s="3"/>
@@ -4243,12 +3473,8 @@
       <c r="L48" s="3"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
-      <c r="A49" t="s" s="0">
-        <v>135</v>
-      </c>
-      <c r="B49" s="31" t="s">
-        <v>136</v>
-      </c>
+      <c r="A49" s="1"/>
+      <c r="B49" s="3"/>
       <c r="D49" s="3"/>
       <c r="E49" s="1"/>
       <c r="F49" s="3"/>
@@ -4259,12 +3485,8 @@
       <c r="L49" s="3"/>
     </row>
     <row r="50" ht="14.25" customHeight="1">
-      <c r="A50" t="s" s="0">
-        <v>137</v>
-      </c>
-      <c r="B50" s="32" t="s">
-        <v>97</v>
-      </c>
+      <c r="A50" s="1"/>
+      <c r="B50" s="3"/>
       <c r="D50" s="3"/>
       <c r="H50" s="3"/>
     </row>
@@ -4755,12 +3977,8 @@
       <c r="F125" s="3"/>
     </row>
     <row r="126" ht="14.25" customHeight="1">
-      <c r="A126" t="s" s="0">
-        <v>138</v>
-      </c>
-      <c r="B126" s="33" t="s">
-        <v>139</v>
-      </c>
+      <c r="A126" s="1"/>
+      <c r="B126" s="3"/>
       <c r="D126" s="3"/>
       <c r="E126" s="1"/>
       <c r="F126" s="3"/>
@@ -5022,12 +4240,7 @@
       <c r="F177" s="3"/>
     </row>
     <row r="178" ht="14.25" customHeight="1">
-      <c r="A178" t="s" s="0">
-        <v>140</v>
-      </c>
-      <c r="B178" s="34" t="s">
-        <v>141</v>
-      </c>
+      <c r="B178" s="3"/>
       <c r="D178" s="3"/>
     </row>
     <row r="179" ht="14.25" customHeight="1">
@@ -5952,12 +5165,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" t="s" s="0">
-        <v>105</v>
-      </c>
-      <c r="B1" s="35" t="s">
-        <v>106</v>
-      </c>
+      <c r="A1" s="1"/>
+      <c r="B1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="1"/>
       <c r="F1" s="3"/>
@@ -5968,12 +5177,8 @@
       <c r="L1" s="3"/>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" t="s" s="0">
-        <v>107</v>
-      </c>
-      <c r="B2" s="36" t="s">
-        <v>29</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="1"/>
       <c r="F2" s="3"/>
@@ -5984,12 +5189,8 @@
       <c r="L2" s="3"/>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" t="s" s="0">
-        <v>142</v>
-      </c>
-      <c r="B3" s="37" t="s">
-        <v>143</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="1"/>
       <c r="F3" s="3"/>
@@ -6000,12 +5201,8 @@
       <c r="L3" s="3"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" t="s" s="0">
-        <v>144</v>
-      </c>
-      <c r="B4" s="38" t="s">
-        <v>145</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="1"/>
       <c r="F4" s="3"/>
@@ -6016,12 +5213,8 @@
       <c r="L4" s="3"/>
     </row>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" t="s" s="0">
-        <v>146</v>
-      </c>
-      <c r="B5" s="39" t="s">
-        <v>145</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="1"/>
       <c r="F5" s="3"/>
@@ -6032,12 +5225,8 @@
       <c r="L5" s="3"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" t="s" s="0">
-        <v>103</v>
-      </c>
-      <c r="B6" s="40" t="s">
-        <v>104</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="1"/>
       <c r="F6" s="3"/>
@@ -6048,12 +5237,8 @@
       <c r="L6" s="3"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" t="s" s="0">
-        <v>147</v>
-      </c>
-      <c r="B7" s="41" t="s">
-        <v>148</v>
-      </c>
+      <c r="A7" s="1"/>
+      <c r="B7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="1"/>
       <c r="F7" s="3"/>
@@ -6064,12 +5249,8 @@
       <c r="L7" s="3"/>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="A8" t="s" s="0">
-        <v>149</v>
-      </c>
-      <c r="B8" s="42" t="s">
-        <v>145</v>
-      </c>
+      <c r="A8" s="1"/>
+      <c r="B8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="1"/>
       <c r="F8" s="3"/>
@@ -6080,12 +5261,8 @@
       <c r="L8" s="3"/>
     </row>
     <row r="9" ht="14.25" customHeight="1">
-      <c r="A9" t="s" s="0">
-        <v>150</v>
-      </c>
-      <c r="B9" s="43" t="s">
-        <v>127</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="B9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="1"/>
       <c r="F9" s="3"/>
@@ -6096,12 +5273,8 @@
       <c r="L9" s="3"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
-      <c r="A10" t="s" s="0">
-        <v>151</v>
-      </c>
-      <c r="B10" s="44" t="s">
-        <v>152</v>
-      </c>
+      <c r="A10" s="1"/>
+      <c r="B10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="1"/>
       <c r="F10" s="3"/>
@@ -6112,12 +5285,8 @@
       <c r="L10" s="3"/>
     </row>
     <row r="11" ht="14.25" customHeight="1">
-      <c r="A11" t="s" s="0">
-        <v>108</v>
-      </c>
-      <c r="B11" s="45" t="s">
-        <v>109</v>
-      </c>
+      <c r="A11" s="1"/>
+      <c r="B11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="1"/>
       <c r="F11" s="3"/>
@@ -6128,12 +5297,8 @@
       <c r="L11" s="3"/>
     </row>
     <row r="12" ht="14.25" customHeight="1">
-      <c r="A12" t="s" s="0">
-        <v>110</v>
-      </c>
-      <c r="B12" s="46" t="s">
-        <v>111</v>
-      </c>
+      <c r="A12" s="1"/>
+      <c r="B12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="1"/>
       <c r="F12" s="3"/>
@@ -6144,12 +5309,8 @@
       <c r="L12" s="3"/>
     </row>
     <row r="13" ht="33" customHeight="1">
-      <c r="A13" t="s" s="0">
-        <v>112</v>
-      </c>
-      <c r="B13" s="47" t="s">
-        <v>153</v>
-      </c>
+      <c r="A13" s="1"/>
+      <c r="B13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="1"/>
       <c r="F13" s="3"/>
@@ -6160,12 +5321,8 @@
       <c r="L13" s="3"/>
     </row>
     <row r="14" ht="14.25" customHeight="1">
-      <c r="A14" t="s" s="0">
-        <v>154</v>
-      </c>
-      <c r="B14" s="48" t="s">
-        <v>152</v>
-      </c>
+      <c r="A14" s="1"/>
+      <c r="B14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="1"/>
       <c r="F14" s="3"/>
@@ -6176,12 +5333,8 @@
       <c r="L14" s="3"/>
     </row>
     <row r="15" ht="14.25" customHeight="1">
-      <c r="A15" t="s" s="0">
-        <v>114</v>
-      </c>
-      <c r="B15" s="49" t="s">
-        <v>115</v>
-      </c>
+      <c r="A15" s="1"/>
+      <c r="B15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="1"/>
       <c r="F15" s="3"/>
@@ -6192,12 +5345,8 @@
       <c r="L15" s="3"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="A16" t="s" s="0">
-        <v>116</v>
-      </c>
-      <c r="B16" s="50" t="s">
-        <v>117</v>
-      </c>
+      <c r="A16" s="1"/>
+      <c r="B16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="1"/>
       <c r="F16" s="3"/>
@@ -6208,12 +5357,8 @@
       <c r="L16" s="3"/>
     </row>
     <row r="17" ht="14.25" customHeight="1">
-      <c r="A17" t="s" s="0">
-        <v>118</v>
-      </c>
-      <c r="B17" s="51" t="s">
-        <v>119</v>
-      </c>
+      <c r="A17" s="1"/>
+      <c r="B17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="1"/>
       <c r="F17" s="3"/>
@@ -6224,12 +5369,8 @@
       <c r="L17" s="3"/>
     </row>
     <row r="18" ht="14.25" customHeight="1">
-      <c r="A18" t="s" s="0">
-        <v>120</v>
-      </c>
-      <c r="B18" s="52" t="s">
-        <v>121</v>
-      </c>
+      <c r="A18" s="1"/>
+      <c r="B18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="1"/>
       <c r="F18" s="3"/>
@@ -6240,12 +5381,8 @@
       <c r="L18" s="3"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" t="s" s="0">
-        <v>122</v>
-      </c>
-      <c r="B19" s="53" t="s">
-        <v>123</v>
-      </c>
+      <c r="A19" s="1"/>
+      <c r="B19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="1"/>
       <c r="F19" s="3"/>
@@ -6256,12 +5393,8 @@
       <c r="L19" s="3"/>
     </row>
     <row r="20" ht="14.25" customHeight="1">
-      <c r="A20" t="s" s="0">
-        <v>155</v>
-      </c>
-      <c r="B20" s="54" t="s">
-        <v>152</v>
-      </c>
+      <c r="A20" s="1"/>
+      <c r="B20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="1"/>
       <c r="F20" s="3"/>
@@ -6272,12 +5405,8 @@
       <c r="L20" s="3"/>
     </row>
     <row r="21" ht="14.25" customHeight="1">
-      <c r="A21" t="s" s="0">
-        <v>124</v>
-      </c>
-      <c r="B21" s="55" t="s">
-        <v>125</v>
-      </c>
+      <c r="A21" s="1"/>
+      <c r="B21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="1"/>
       <c r="F21" s="3"/>
@@ -6288,12 +5417,8 @@
       <c r="L21" s="3"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
-      <c r="A22" t="s" s="0">
-        <v>126</v>
-      </c>
-      <c r="B22" s="56" t="s">
-        <v>127</v>
-      </c>
+      <c r="A22" s="1"/>
+      <c r="B22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="1"/>
       <c r="F22" s="3"/>
@@ -6304,12 +5429,8 @@
       <c r="L22" s="3"/>
     </row>
     <row r="23" ht="14.25" customHeight="1">
-      <c r="A23" t="s" s="0">
-        <v>156</v>
-      </c>
-      <c r="B23" s="57" t="s">
-        <v>157</v>
-      </c>
+      <c r="A23" s="1"/>
+      <c r="B23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="1"/>
       <c r="F23" s="3"/>
@@ -6320,12 +5441,8 @@
       <c r="L23" s="3"/>
     </row>
     <row r="24" ht="14.25" customHeight="1">
-      <c r="A24" t="s" s="0">
-        <v>133</v>
-      </c>
-      <c r="B24" s="58" t="s">
-        <v>158</v>
-      </c>
+      <c r="A24" s="1"/>
+      <c r="B24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="1"/>
       <c r="F24" s="3"/>
@@ -6336,12 +5453,8 @@
       <c r="L24" s="3"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
-      <c r="A25" t="s" s="0">
-        <v>159</v>
-      </c>
-      <c r="B25" s="59" t="s">
-        <v>160</v>
-      </c>
+      <c r="A25" s="1"/>
+      <c r="B25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="1"/>
       <c r="F25" s="3"/>
@@ -6352,12 +5465,8 @@
       <c r="L25" s="3"/>
     </row>
     <row r="26" ht="14.25" customHeight="1">
-      <c r="A26" t="s" s="0">
-        <v>161</v>
-      </c>
-      <c r="B26" s="60" t="s">
-        <v>129</v>
-      </c>
+      <c r="A26" s="1"/>
+      <c r="B26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="1"/>
       <c r="F26" s="3"/>
@@ -6368,12 +5477,8 @@
       <c r="L26" s="3"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
-      <c r="A27" t="s" s="0">
-        <v>130</v>
-      </c>
-      <c r="B27" s="61" t="s">
-        <v>79</v>
-      </c>
+      <c r="A27" s="1"/>
+      <c r="B27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="1"/>
       <c r="F27" s="3"/>
@@ -6384,12 +5489,8 @@
       <c r="L27" s="3"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
-      <c r="A28" t="s" s="0">
-        <v>131</v>
-      </c>
-      <c r="B28" s="62" t="s">
-        <v>132</v>
-      </c>
+      <c r="A28" s="1"/>
+      <c r="B28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="1"/>
       <c r="F28" s="3"/>
@@ -6400,12 +5501,8 @@
       <c r="L28" s="3"/>
     </row>
     <row r="29" ht="14.25" customHeight="1">
-      <c r="A29" t="s" s="0">
-        <v>133</v>
-      </c>
-      <c r="B29" s="63" t="s">
-        <v>134</v>
-      </c>
+      <c r="A29" s="1"/>
+      <c r="B29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="1"/>
       <c r="F29" s="3"/>
@@ -6416,12 +5513,8 @@
       <c r="L29" s="3"/>
     </row>
     <row r="30" ht="14.25" customHeight="1">
-      <c r="A30" t="s" s="0">
-        <v>135</v>
-      </c>
-      <c r="B30" s="64" t="s">
-        <v>136</v>
-      </c>
+      <c r="A30" s="1"/>
+      <c r="B30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="1"/>
       <c r="F30" s="3"/>
@@ -6432,12 +5525,8 @@
       <c r="L30" s="3"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
-      <c r="A31" t="s" s="0">
-        <v>137</v>
-      </c>
-      <c r="B31" s="65" t="s">
-        <v>97</v>
-      </c>
+      <c r="A31" s="1"/>
+      <c r="B31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="1"/>
       <c r="F31" s="3"/>
@@ -8142,12 +7231,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" t="s" s="0">
-        <v>105</v>
-      </c>
-      <c r="B1" s="66" t="s">
-        <v>106</v>
-      </c>
+      <c r="A1" s="1"/>
+      <c r="B1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="1"/>
       <c r="F1" s="3"/>
@@ -8158,12 +7243,8 @@
       <c r="L1" s="3"/>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" t="s" s="0">
-        <v>107</v>
-      </c>
-      <c r="B2" s="67" t="s">
-        <v>29</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="1"/>
       <c r="F2" s="3"/>
@@ -8174,12 +7255,8 @@
       <c r="L2" s="3"/>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" t="s" s="0">
-        <v>142</v>
-      </c>
-      <c r="B3" s="68" t="s">
-        <v>143</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="1"/>
       <c r="F3" s="3"/>
@@ -8190,12 +7267,8 @@
       <c r="L3" s="3"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" t="s" s="0">
-        <v>144</v>
-      </c>
-      <c r="B4" s="69" t="s">
-        <v>145</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="1"/>
       <c r="F4" s="3"/>
@@ -8206,12 +7279,8 @@
       <c r="L4" s="3"/>
     </row>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" t="s" s="0">
-        <v>146</v>
-      </c>
-      <c r="B5" s="70" t="s">
-        <v>145</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="1"/>
       <c r="F5" s="3"/>
@@ -8222,12 +7291,8 @@
       <c r="L5" s="3"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" t="s" s="0">
-        <v>103</v>
-      </c>
-      <c r="B6" s="71" t="s">
-        <v>104</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="1"/>
       <c r="F6" s="3"/>
@@ -8238,12 +7303,8 @@
       <c r="L6" s="3"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" t="s" s="0">
-        <v>147</v>
-      </c>
-      <c r="B7" s="72" t="s">
-        <v>148</v>
-      </c>
+      <c r="A7" s="1"/>
+      <c r="B7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="1"/>
       <c r="F7" s="3"/>
@@ -8254,12 +7315,8 @@
       <c r="L7" s="3"/>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="A8" t="s" s="0">
-        <v>149</v>
-      </c>
-      <c r="B8" s="73" t="s">
-        <v>145</v>
-      </c>
+      <c r="A8" s="1"/>
+      <c r="B8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="1"/>
       <c r="F8" s="3"/>
@@ -8270,12 +7327,8 @@
       <c r="L8" s="3"/>
     </row>
     <row r="9" ht="14.25" customHeight="1">
-      <c r="A9" t="s" s="0">
-        <v>150</v>
-      </c>
-      <c r="B9" s="74" t="s">
-        <v>127</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="B9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="1"/>
       <c r="F9" s="3"/>
@@ -8286,12 +7339,8 @@
       <c r="L9" s="3"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
-      <c r="A10" t="s" s="0">
-        <v>151</v>
-      </c>
-      <c r="B10" s="75" t="s">
-        <v>152</v>
-      </c>
+      <c r="A10" s="1"/>
+      <c r="B10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="1"/>
       <c r="F10" s="3"/>
@@ -8302,12 +7351,8 @@
       <c r="L10" s="3"/>
     </row>
     <row r="11" ht="14.25" customHeight="1">
-      <c r="A11" t="s" s="0">
-        <v>108</v>
-      </c>
-      <c r="B11" s="76" t="s">
-        <v>109</v>
-      </c>
+      <c r="A11" s="1"/>
+      <c r="B11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="1"/>
       <c r="F11" s="3"/>
@@ -8318,12 +7363,8 @@
       <c r="L11" s="3"/>
     </row>
     <row r="12" ht="14.25" customHeight="1">
-      <c r="A12" t="s" s="0">
-        <v>110</v>
-      </c>
-      <c r="B12" s="77" t="s">
-        <v>111</v>
-      </c>
+      <c r="A12" s="1"/>
+      <c r="B12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="1"/>
       <c r="F12" s="3"/>
@@ -8334,12 +7375,8 @@
       <c r="L12" s="3"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
-      <c r="A13" t="s" s="0">
-        <v>112</v>
-      </c>
-      <c r="B13" s="78" t="s">
-        <v>153</v>
-      </c>
+      <c r="A13" s="1"/>
+      <c r="B13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="1"/>
       <c r="F13" s="3"/>
@@ -8350,12 +7387,8 @@
       <c r="L13" s="3"/>
     </row>
     <row r="14" ht="14.25" customHeight="1">
-      <c r="A14" t="s" s="0">
-        <v>154</v>
-      </c>
-      <c r="B14" s="79" t="s">
-        <v>152</v>
-      </c>
+      <c r="A14" s="1"/>
+      <c r="B14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="1"/>
       <c r="F14" s="3"/>
@@ -8366,12 +7399,8 @@
       <c r="L14" s="3"/>
     </row>
     <row r="15" ht="14.25" customHeight="1">
-      <c r="A15" t="s" s="0">
-        <v>114</v>
-      </c>
-      <c r="B15" s="80" t="s">
-        <v>115</v>
-      </c>
+      <c r="A15" s="1"/>
+      <c r="B15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="1"/>
       <c r="F15" s="3"/>
@@ -8382,12 +7411,8 @@
       <c r="L15" s="3"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="A16" t="s" s="0">
-        <v>116</v>
-      </c>
-      <c r="B16" s="81" t="s">
-        <v>117</v>
-      </c>
+      <c r="A16" s="1"/>
+      <c r="B16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="1"/>
       <c r="F16" s="3"/>
@@ -8398,12 +7423,8 @@
       <c r="L16" s="3"/>
     </row>
     <row r="17" ht="14.25" customHeight="1">
-      <c r="A17" t="s" s="0">
-        <v>118</v>
-      </c>
-      <c r="B17" s="82" t="s">
-        <v>119</v>
-      </c>
+      <c r="A17" s="1"/>
+      <c r="B17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="1"/>
       <c r="F17" s="3"/>
@@ -8414,12 +7435,8 @@
       <c r="L17" s="3"/>
     </row>
     <row r="18" ht="14.25" customHeight="1">
-      <c r="A18" t="s" s="0">
-        <v>120</v>
-      </c>
-      <c r="B18" s="83" t="s">
-        <v>121</v>
-      </c>
+      <c r="A18" s="1"/>
+      <c r="B18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="1"/>
       <c r="F18" s="3"/>
@@ -8430,12 +7447,8 @@
       <c r="L18" s="3"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" t="s" s="0">
-        <v>122</v>
-      </c>
-      <c r="B19" s="84" t="s">
-        <v>123</v>
-      </c>
+      <c r="A19" s="1"/>
+      <c r="B19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="1"/>
       <c r="F19" s="3"/>
@@ -8446,12 +7459,8 @@
       <c r="L19" s="3"/>
     </row>
     <row r="20" ht="14.25" customHeight="1">
-      <c r="A20" t="s" s="0">
-        <v>155</v>
-      </c>
-      <c r="B20" s="85" t="s">
-        <v>152</v>
-      </c>
+      <c r="A20" s="1"/>
+      <c r="B20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="1"/>
       <c r="F20" s="3"/>
@@ -8462,12 +7471,8 @@
       <c r="L20" s="3"/>
     </row>
     <row r="21" ht="14.25" customHeight="1">
-      <c r="A21" t="s" s="0">
-        <v>124</v>
-      </c>
-      <c r="B21" s="86" t="s">
-        <v>125</v>
-      </c>
+      <c r="A21" s="1"/>
+      <c r="B21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="1"/>
       <c r="F21" s="3"/>
@@ -8478,12 +7483,8 @@
       <c r="L21" s="3"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
-      <c r="A22" t="s" s="0">
-        <v>126</v>
-      </c>
-      <c r="B22" s="87" t="s">
-        <v>127</v>
-      </c>
+      <c r="A22" s="1"/>
+      <c r="B22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="1"/>
       <c r="F22" s="3"/>
@@ -8494,12 +7495,8 @@
       <c r="L22" s="3"/>
     </row>
     <row r="23" ht="14.25" customHeight="1">
-      <c r="A23" t="s" s="0">
-        <v>156</v>
-      </c>
-      <c r="B23" s="88" t="s">
-        <v>157</v>
-      </c>
+      <c r="A23" s="1"/>
+      <c r="B23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="1"/>
       <c r="F23" s="3"/>
@@ -8510,12 +7507,8 @@
       <c r="L23" s="3"/>
     </row>
     <row r="24" ht="14.25" customHeight="1">
-      <c r="A24" t="s" s="0">
-        <v>133</v>
-      </c>
-      <c r="B24" s="89" t="s">
-        <v>158</v>
-      </c>
+      <c r="A24" s="1"/>
+      <c r="B24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="1"/>
       <c r="F24" s="3"/>
@@ -8526,12 +7519,8 @@
       <c r="L24" s="3"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
-      <c r="A25" t="s" s="0">
-        <v>159</v>
-      </c>
-      <c r="B25" s="90" t="s">
-        <v>160</v>
-      </c>
+      <c r="A25" s="1"/>
+      <c r="B25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="1"/>
       <c r="F25" s="3"/>
@@ -8542,12 +7531,8 @@
       <c r="L25" s="3"/>
     </row>
     <row r="26" ht="14.25" customHeight="1">
-      <c r="A26" t="s" s="0">
-        <v>161</v>
-      </c>
-      <c r="B26" s="91" t="s">
-        <v>129</v>
-      </c>
+      <c r="A26" s="1"/>
+      <c r="B26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="1"/>
       <c r="F26" s="3"/>
@@ -8558,12 +7543,8 @@
       <c r="L26" s="3"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
-      <c r="A27" t="s" s="0">
-        <v>130</v>
-      </c>
-      <c r="B27" s="92" t="s">
-        <v>79</v>
-      </c>
+      <c r="A27" s="1"/>
+      <c r="B27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="1"/>
       <c r="F27" s="3"/>
@@ -8574,12 +7555,8 @@
       <c r="L27" s="3"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
-      <c r="A28" t="s" s="0">
-        <v>131</v>
-      </c>
-      <c r="B28" s="93" t="s">
-        <v>132</v>
-      </c>
+      <c r="A28" s="1"/>
+      <c r="B28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="1"/>
       <c r="F28" s="3"/>
@@ -8590,12 +7567,8 @@
       <c r="L28" s="3"/>
     </row>
     <row r="29" ht="14.25" customHeight="1">
-      <c r="A29" t="s" s="0">
-        <v>133</v>
-      </c>
-      <c r="B29" s="94" t="s">
-        <v>134</v>
-      </c>
+      <c r="A29" s="1"/>
+      <c r="B29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="1"/>
       <c r="F29" s="3"/>
@@ -8606,12 +7579,8 @@
       <c r="L29" s="3"/>
     </row>
     <row r="30" ht="14.25" customHeight="1">
-      <c r="A30" t="s" s="0">
-        <v>135</v>
-      </c>
-      <c r="B30" s="95" t="s">
-        <v>136</v>
-      </c>
+      <c r="A30" s="1"/>
+      <c r="B30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="1"/>
       <c r="F30" s="3"/>
@@ -8622,12 +7591,8 @@
       <c r="L30" s="3"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
-      <c r="A31" t="s" s="0">
-        <v>137</v>
-      </c>
-      <c r="B31" s="96" t="s">
-        <v>97</v>
-      </c>
+      <c r="A31" s="1"/>
+      <c r="B31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="1"/>
       <c r="F31" s="3"/>
@@ -8638,12 +7603,8 @@
       <c r="L31" s="3"/>
     </row>
     <row r="32" ht="14.25" customHeight="1">
-      <c r="A32" t="s" s="0">
-        <v>138</v>
-      </c>
-      <c r="B32" s="97" t="s">
-        <v>139</v>
-      </c>
+      <c r="A32" s="1"/>
+      <c r="B32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="1"/>
       <c r="F32" s="3"/>
@@ -8654,12 +7615,8 @@
       <c r="L32" s="3"/>
     </row>
     <row r="33" ht="14.25" customHeight="1">
-      <c r="A33" t="s" s="0">
-        <v>165</v>
-      </c>
-      <c r="B33" s="98" t="s">
-        <v>141</v>
-      </c>
+      <c r="A33" s="1"/>
+      <c r="B33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="1"/>
       <c r="F33" s="3"/>

</xml_diff>

<commit_message>
Till Pre app dashboard page Xpaths updates
</commit_message>
<xml_diff>
--- a/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
+++ b/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>TCID</t>
   </si>
@@ -340,28 +340,12 @@
   </si>
   <si>
     <t>Test Degree</t>
-  </si>
-  <si>
-    <t>Legal name</t>
-  </si>
-  <si>
-    <t>Test FN Automation MN Test LN</t>
-  </si>
-  <si>
-    <t>Preferred first name</t>
-  </si>
-  <si>
-    <t>Date of birth</t>
-  </si>
-  <si>
-    <t>November 13, 1964</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="9">
     <font>
       <sz val="11"/>
@@ -433,7 +417,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -456,15 +440,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -673,11 +648,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="24.57"/>
-    <col min="2" max="6" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="24.57" customWidth="1"/>
+    <col min="2" max="6" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2391,15 +2365,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="38.29"/>
-    <col min="3" max="3" customWidth="true" width="34.0"/>
-    <col min="4" max="4" customWidth="true" width="22.29"/>
-    <col min="5" max="5" customWidth="true" width="30.0"/>
-    <col min="6" max="6" customWidth="true" width="18.57"/>
-    <col min="7" max="7" customWidth="true" width="30.14"/>
+    <col min="1" max="2" width="38.29" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="22.29" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="18.57" customWidth="1"/>
+    <col min="7" max="7" width="30.14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2491,14 +2464,13 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="38.29"/>
-    <col min="3" max="3" customWidth="true" width="34.0"/>
-    <col min="4" max="4" customWidth="true" width="22.29"/>
-    <col min="5" max="5" customWidth="true" width="30.0"/>
-    <col min="6" max="6" customWidth="true" width="14.43"/>
+    <col min="1" max="2" width="38.29" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="22.29" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2572,14 +2544,13 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.14"/>
-    <col min="2" max="2" customWidth="true" width="29.57"/>
-    <col min="3" max="3" customWidth="true" width="41.43"/>
-    <col min="4" max="4" customWidth="true" width="34.43"/>
-    <col min="5" max="5" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="27.14" customWidth="1"/>
+    <col min="2" max="2" width="29.57" customWidth="1"/>
+    <col min="3" max="3" width="41.43" customWidth="1"/>
+    <col min="4" max="4" width="34.43" customWidth="1"/>
+    <col min="5" max="5" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2644,10 +2615,9 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="5" customWidth="true" width="14.43"/>
+    <col min="1" max="5" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2831,10 +2801,9 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="4" customWidth="true" width="14.43"/>
+    <col min="1" max="4" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2928,14 +2897,13 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="31.0"/>
-    <col min="2" max="2" customWidth="true" width="27.43"/>
-    <col min="3" max="3" customWidth="true" width="51.0"/>
-    <col min="4" max="4" customWidth="true" width="22.43"/>
-    <col min="5" max="5" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="31" customWidth="1"/>
+    <col min="2" max="2" width="27.43" customWidth="1"/>
+    <col min="3" max="3" width="51" customWidth="1"/>
+    <col min="4" max="4" width="22.43" customWidth="1"/>
+    <col min="5" max="5" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2997,17 +2965,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="36.86"/>
-    <col min="2" max="2" customWidth="true" width="41.14"/>
-    <col min="3" max="3" customWidth="true" width="20.43"/>
-    <col min="4" max="4" customWidth="true" width="20.14"/>
-    <col min="5" max="5" customWidth="true" width="31.43"/>
-    <col min="6" max="6" customWidth="true" width="24.43"/>
-    <col min="7" max="7" customWidth="true" width="26.71"/>
-    <col min="12" max="12" customWidth="true" width="40.71"/>
+    <col min="1" max="1" width="36.86" customWidth="1"/>
+    <col min="2" max="2" width="41.14" customWidth="1"/>
+    <col min="3" max="3" width="20.43" customWidth="1"/>
+    <col min="4" max="4" width="20.14" customWidth="1"/>
+    <col min="5" max="5" width="31.43" customWidth="1"/>
+    <col min="6" max="6" width="24.43" customWidth="1"/>
+    <col min="7" max="7" width="26.71" customWidth="1"/>
+    <col min="12" max="12" width="40.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -3021,12 +2988,8 @@
       <c r="L1" s="3"/>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" t="s" s="0">
-        <v>103</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>104</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="1"/>
       <c r="F2" s="3"/>
@@ -3035,12 +2998,8 @@
       <c r="L2" s="3"/>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" t="s" s="0">
-        <v>105</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>29</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="1"/>
       <c r="F3" s="3"/>
@@ -3049,12 +3008,8 @@
       <c r="L3" s="3"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" t="s" s="0">
-        <v>106</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>107</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="1"/>
       <c r="F4" s="3"/>
@@ -5153,15 +5108,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="13.14"/>
-    <col min="2" max="2" customWidth="true" width="23.71"/>
-    <col min="3" max="3" customWidth="true" width="45.14"/>
-    <col min="4" max="4" customWidth="true" width="14.57"/>
-    <col min="5" max="5" customWidth="true" width="60.0"/>
-    <col min="6" max="6" customWidth="true" width="25.14"/>
+    <col min="1" max="1" width="13.14" customWidth="1"/>
+    <col min="2" max="2" width="23.71" customWidth="1"/>
+    <col min="3" max="3" width="45.14" customWidth="1"/>
+    <col min="4" max="4" width="14.57" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
+    <col min="6" max="6" width="25.14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -7219,15 +7173,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="37.29"/>
-    <col min="2" max="2" customWidth="true" width="29.57"/>
-    <col min="3" max="3" customWidth="true" width="24.57"/>
-    <col min="4" max="4" customWidth="true" width="27.57"/>
-    <col min="5" max="5" customWidth="true" width="25.29"/>
-    <col min="6" max="6" customWidth="true" width="33.57"/>
+    <col min="1" max="1" width="37.29" customWidth="1"/>
+    <col min="2" max="2" width="29.57" customWidth="1"/>
+    <col min="3" max="3" width="24.57" customWidth="1"/>
+    <col min="4" max="4" width="27.57" customWidth="1"/>
+    <col min="5" max="5" width="25.29" customWidth="1"/>
+    <col min="6" max="6" width="33.57" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9281,12 +9234,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.29"/>
-    <col min="2" max="2" customWidth="true" width="14.14"/>
-    <col min="3" max="3" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="27.29" customWidth="1"/>
+    <col min="2" max="2" width="14.14" customWidth="1"/>
+    <col min="3" max="3" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9344,14 +9296,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="29.43"/>
-    <col min="2" max="2" customWidth="true" width="31.43"/>
-    <col min="3" max="3" customWidth="true" width="28.71"/>
-    <col min="4" max="4" customWidth="true" width="30.57"/>
-    <col min="5" max="5" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="29.43" customWidth="1"/>
+    <col min="2" max="2" width="31.43" customWidth="1"/>
+    <col min="3" max="3" width="28.71" customWidth="1"/>
+    <col min="4" max="4" width="30.57" customWidth="1"/>
+    <col min="5" max="5" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9464,13 +9415,12 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.29"/>
-    <col min="2" max="2" customWidth="true" width="20.14"/>
-    <col min="3" max="4" customWidth="true" width="13.57"/>
-    <col min="5" max="5" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="27.29" customWidth="1"/>
+    <col min="2" max="2" width="20.14" customWidth="1"/>
+    <col min="3" max="4" width="13.57" customWidth="1"/>
+    <col min="5" max="5" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9569,12 +9519,11 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.57"/>
-    <col min="2" max="2" customWidth="true" width="39.86"/>
-    <col min="3" max="3" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="27.57" customWidth="1"/>
+    <col min="2" max="2" width="39.86" customWidth="1"/>
+    <col min="3" max="3" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9753,12 +9702,11 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="56.0"/>
-    <col min="2" max="2" customWidth="true" width="57.0"/>
-    <col min="3" max="3" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="56" customWidth="1"/>
+    <col min="2" max="2" width="57" customWidth="1"/>
+    <col min="3" max="3" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Preapp dashboard xpaths upadted
</commit_message>
<xml_diff>
--- a/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
+++ b/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>TCID</t>
   </si>
@@ -340,12 +340,28 @@
   </si>
   <si>
     <t>Test Degree</t>
+  </si>
+  <si>
+    <t>Legal name</t>
+  </si>
+  <si>
+    <t>Test FN Automation MN Test LN</t>
+  </si>
+  <si>
+    <t>Preferred first name</t>
+  </si>
+  <si>
+    <t>Date of birth</t>
+  </si>
+  <si>
+    <t>January 23, 1962</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="9">
     <font>
       <sz val="11"/>
@@ -417,7 +433,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -440,6 +456,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -648,10 +673,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="24.57" customWidth="1"/>
-    <col min="2" max="6" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="24.57"/>
+    <col min="2" max="6" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2365,14 +2391,15 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="38.29" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="22.29" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="18.57" customWidth="1"/>
-    <col min="7" max="7" width="30.14" customWidth="1"/>
+    <col min="1" max="2" customWidth="true" width="38.29"/>
+    <col min="3" max="3" customWidth="true" width="34.0"/>
+    <col min="4" max="4" customWidth="true" width="22.29"/>
+    <col min="5" max="5" customWidth="true" width="30.0"/>
+    <col min="6" max="6" customWidth="true" width="18.57"/>
+    <col min="7" max="7" customWidth="true" width="30.14"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2464,13 +2491,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="38.29" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="22.29" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="14.43" customWidth="1"/>
+    <col min="1" max="2" customWidth="true" width="38.29"/>
+    <col min="3" max="3" customWidth="true" width="34.0"/>
+    <col min="4" max="4" customWidth="true" width="22.29"/>
+    <col min="5" max="5" customWidth="true" width="30.0"/>
+    <col min="6" max="6" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2544,13 +2572,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.14" customWidth="1"/>
-    <col min="2" max="2" width="29.57" customWidth="1"/>
-    <col min="3" max="3" width="41.43" customWidth="1"/>
-    <col min="4" max="4" width="34.43" customWidth="1"/>
-    <col min="5" max="5" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.14"/>
+    <col min="2" max="2" customWidth="true" width="29.57"/>
+    <col min="3" max="3" customWidth="true" width="41.43"/>
+    <col min="4" max="4" customWidth="true" width="34.43"/>
+    <col min="5" max="5" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2615,9 +2644,10 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="14.43" customWidth="1"/>
+    <col min="1" max="5" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2801,9 +2831,10 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="4" width="14.43" customWidth="1"/>
+    <col min="1" max="4" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2897,13 +2928,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31" customWidth="1"/>
-    <col min="2" max="2" width="27.43" customWidth="1"/>
-    <col min="3" max="3" width="51" customWidth="1"/>
-    <col min="4" max="4" width="22.43" customWidth="1"/>
-    <col min="5" max="5" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="31.0"/>
+    <col min="2" max="2" customWidth="true" width="27.43"/>
+    <col min="3" max="3" customWidth="true" width="51.0"/>
+    <col min="4" max="4" customWidth="true" width="22.43"/>
+    <col min="5" max="5" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2965,16 +2997,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="36.86" customWidth="1"/>
-    <col min="2" max="2" width="41.14" customWidth="1"/>
-    <col min="3" max="3" width="20.43" customWidth="1"/>
-    <col min="4" max="4" width="20.14" customWidth="1"/>
-    <col min="5" max="5" width="31.43" customWidth="1"/>
-    <col min="6" max="6" width="24.43" customWidth="1"/>
-    <col min="7" max="7" width="26.71" customWidth="1"/>
-    <col min="12" max="12" width="40.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="36.86"/>
+    <col min="2" max="2" customWidth="true" width="41.14"/>
+    <col min="3" max="3" customWidth="true" width="20.43"/>
+    <col min="4" max="4" customWidth="true" width="20.14"/>
+    <col min="5" max="5" customWidth="true" width="31.43"/>
+    <col min="6" max="6" customWidth="true" width="24.43"/>
+    <col min="7" max="7" customWidth="true" width="26.71"/>
+    <col min="12" max="12" customWidth="true" width="40.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -2988,8 +3021,12 @@
       <c r="L1" s="3"/>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="1"/>
-      <c r="B2" s="3"/>
+      <c r="A2" t="s" s="0">
+        <v>103</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>104</v>
+      </c>
       <c r="D2" s="3"/>
       <c r="E2" s="1"/>
       <c r="F2" s="3"/>
@@ -2998,8 +3035,12 @@
       <c r="L2" s="3"/>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" s="1"/>
-      <c r="B3" s="3"/>
+      <c r="A3" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>29</v>
+      </c>
       <c r="D3" s="3"/>
       <c r="E3" s="1"/>
       <c r="F3" s="3"/>
@@ -3008,8 +3049,12 @@
       <c r="L3" s="3"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" s="1"/>
-      <c r="B4" s="3"/>
+      <c r="A4" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>107</v>
+      </c>
       <c r="D4" s="3"/>
       <c r="E4" s="1"/>
       <c r="F4" s="3"/>
@@ -5108,14 +5153,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.14" customWidth="1"/>
-    <col min="2" max="2" width="23.71" customWidth="1"/>
-    <col min="3" max="3" width="45.14" customWidth="1"/>
-    <col min="4" max="4" width="14.57" customWidth="1"/>
-    <col min="5" max="5" width="60" customWidth="1"/>
-    <col min="6" max="6" width="25.14" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="13.14"/>
+    <col min="2" max="2" customWidth="true" width="23.71"/>
+    <col min="3" max="3" customWidth="true" width="45.14"/>
+    <col min="4" max="4" customWidth="true" width="14.57"/>
+    <col min="5" max="5" customWidth="true" width="60.0"/>
+    <col min="6" max="6" customWidth="true" width="25.14"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -7173,14 +7219,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="37.29" customWidth="1"/>
-    <col min="2" max="2" width="29.57" customWidth="1"/>
-    <col min="3" max="3" width="24.57" customWidth="1"/>
-    <col min="4" max="4" width="27.57" customWidth="1"/>
-    <col min="5" max="5" width="25.29" customWidth="1"/>
-    <col min="6" max="6" width="33.57" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="37.29"/>
+    <col min="2" max="2" customWidth="true" width="29.57"/>
+    <col min="3" max="3" customWidth="true" width="24.57"/>
+    <col min="4" max="4" customWidth="true" width="27.57"/>
+    <col min="5" max="5" customWidth="true" width="25.29"/>
+    <col min="6" max="6" customWidth="true" width="33.57"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9234,11 +9281,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.29" customWidth="1"/>
-    <col min="2" max="2" width="14.14" customWidth="1"/>
-    <col min="3" max="3" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.29"/>
+    <col min="2" max="2" customWidth="true" width="14.14"/>
+    <col min="3" max="3" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9296,13 +9344,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="29.43" customWidth="1"/>
-    <col min="2" max="2" width="31.43" customWidth="1"/>
-    <col min="3" max="3" width="28.71" customWidth="1"/>
-    <col min="4" max="4" width="30.57" customWidth="1"/>
-    <col min="5" max="5" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="29.43"/>
+    <col min="2" max="2" customWidth="true" width="31.43"/>
+    <col min="3" max="3" customWidth="true" width="28.71"/>
+    <col min="4" max="4" customWidth="true" width="30.57"/>
+    <col min="5" max="5" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9415,12 +9464,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.29" customWidth="1"/>
-    <col min="2" max="2" width="20.14" customWidth="1"/>
-    <col min="3" max="4" width="13.57" customWidth="1"/>
-    <col min="5" max="5" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.29"/>
+    <col min="2" max="2" customWidth="true" width="20.14"/>
+    <col min="3" max="4" customWidth="true" width="13.57"/>
+    <col min="5" max="5" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9519,11 +9569,12 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.57" customWidth="1"/>
-    <col min="2" max="2" width="39.86" customWidth="1"/>
-    <col min="3" max="3" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.57"/>
+    <col min="2" max="2" customWidth="true" width="39.86"/>
+    <col min="3" max="3" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9702,11 +9753,12 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="56" customWidth="1"/>
-    <col min="2" max="2" width="57" customWidth="1"/>
-    <col min="3" max="3" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="56.0"/>
+    <col min="2" max="2" customWidth="true" width="57.0"/>
+    <col min="3" max="3" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Latest code - My Info - In progress
</commit_message>
<xml_diff>
--- a/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
+++ b/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>TCID</t>
   </si>
@@ -340,28 +340,12 @@
   </si>
   <si>
     <t>Test Degree</t>
-  </si>
-  <si>
-    <t>Legal name</t>
-  </si>
-  <si>
-    <t>Test FN Automation MN Test LN</t>
-  </si>
-  <si>
-    <t>Preferred first name</t>
-  </si>
-  <si>
-    <t>Date of birth</t>
-  </si>
-  <si>
-    <t>January 23, 1962</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="9">
     <font>
       <sz val="11"/>
@@ -433,7 +417,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -456,15 +440,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -673,11 +648,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="24.57"/>
-    <col min="2" max="6" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="24.57" customWidth="1"/>
+    <col min="2" max="6" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2391,15 +2365,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="38.29"/>
-    <col min="3" max="3" customWidth="true" width="34.0"/>
-    <col min="4" max="4" customWidth="true" width="22.29"/>
-    <col min="5" max="5" customWidth="true" width="30.0"/>
-    <col min="6" max="6" customWidth="true" width="18.57"/>
-    <col min="7" max="7" customWidth="true" width="30.14"/>
+    <col min="1" max="2" width="38.29" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="22.29" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="18.57" customWidth="1"/>
+    <col min="7" max="7" width="30.14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2491,14 +2464,13 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="38.29"/>
-    <col min="3" max="3" customWidth="true" width="34.0"/>
-    <col min="4" max="4" customWidth="true" width="22.29"/>
-    <col min="5" max="5" customWidth="true" width="30.0"/>
-    <col min="6" max="6" customWidth="true" width="14.43"/>
+    <col min="1" max="2" width="38.29" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="22.29" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2572,14 +2544,13 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.14"/>
-    <col min="2" max="2" customWidth="true" width="29.57"/>
-    <col min="3" max="3" customWidth="true" width="41.43"/>
-    <col min="4" max="4" customWidth="true" width="34.43"/>
-    <col min="5" max="5" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="27.14" customWidth="1"/>
+    <col min="2" max="2" width="29.57" customWidth="1"/>
+    <col min="3" max="3" width="41.43" customWidth="1"/>
+    <col min="4" max="4" width="34.43" customWidth="1"/>
+    <col min="5" max="5" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2644,10 +2615,9 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="5" customWidth="true" width="14.43"/>
+    <col min="1" max="5" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2831,10 +2801,9 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="4" customWidth="true" width="14.43"/>
+    <col min="1" max="4" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2928,14 +2897,13 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="31.0"/>
-    <col min="2" max="2" customWidth="true" width="27.43"/>
-    <col min="3" max="3" customWidth="true" width="51.0"/>
-    <col min="4" max="4" customWidth="true" width="22.43"/>
-    <col min="5" max="5" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="31" customWidth="1"/>
+    <col min="2" max="2" width="27.43" customWidth="1"/>
+    <col min="3" max="3" width="51" customWidth="1"/>
+    <col min="4" max="4" width="22.43" customWidth="1"/>
+    <col min="5" max="5" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2997,17 +2965,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="36.86"/>
-    <col min="2" max="2" customWidth="true" width="41.14"/>
-    <col min="3" max="3" customWidth="true" width="20.43"/>
-    <col min="4" max="4" customWidth="true" width="20.14"/>
-    <col min="5" max="5" customWidth="true" width="31.43"/>
-    <col min="6" max="6" customWidth="true" width="24.43"/>
-    <col min="7" max="7" customWidth="true" width="26.71"/>
-    <col min="12" max="12" customWidth="true" width="40.71"/>
+    <col min="1" max="1" width="36.86" customWidth="1"/>
+    <col min="2" max="2" width="41.14" customWidth="1"/>
+    <col min="3" max="3" width="20.43" customWidth="1"/>
+    <col min="4" max="4" width="20.14" customWidth="1"/>
+    <col min="5" max="5" width="31.43" customWidth="1"/>
+    <col min="6" max="6" width="24.43" customWidth="1"/>
+    <col min="7" max="7" width="26.71" customWidth="1"/>
+    <col min="12" max="12" width="40.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -3021,12 +2988,8 @@
       <c r="L1" s="3"/>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" t="s" s="0">
-        <v>103</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>104</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="1"/>
       <c r="F2" s="3"/>
@@ -3035,12 +2998,8 @@
       <c r="L2" s="3"/>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" t="s" s="0">
-        <v>105</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>29</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="1"/>
       <c r="F3" s="3"/>
@@ -3049,12 +3008,8 @@
       <c r="L3" s="3"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" t="s" s="0">
-        <v>106</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>107</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="1"/>
       <c r="F4" s="3"/>
@@ -5153,15 +5108,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="13.14"/>
-    <col min="2" max="2" customWidth="true" width="23.71"/>
-    <col min="3" max="3" customWidth="true" width="45.14"/>
-    <col min="4" max="4" customWidth="true" width="14.57"/>
-    <col min="5" max="5" customWidth="true" width="60.0"/>
-    <col min="6" max="6" customWidth="true" width="25.14"/>
+    <col min="1" max="1" width="13.14" customWidth="1"/>
+    <col min="2" max="2" width="23.71" customWidth="1"/>
+    <col min="3" max="3" width="45.14" customWidth="1"/>
+    <col min="4" max="4" width="14.57" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
+    <col min="6" max="6" width="25.14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -7219,15 +7173,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="37.29"/>
-    <col min="2" max="2" customWidth="true" width="29.57"/>
-    <col min="3" max="3" customWidth="true" width="24.57"/>
-    <col min="4" max="4" customWidth="true" width="27.57"/>
-    <col min="5" max="5" customWidth="true" width="25.29"/>
-    <col min="6" max="6" customWidth="true" width="33.57"/>
+    <col min="1" max="1" width="37.29" customWidth="1"/>
+    <col min="2" max="2" width="29.57" customWidth="1"/>
+    <col min="3" max="3" width="24.57" customWidth="1"/>
+    <col min="4" max="4" width="27.57" customWidth="1"/>
+    <col min="5" max="5" width="25.29" customWidth="1"/>
+    <col min="6" max="6" width="33.57" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9281,12 +9234,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.29"/>
-    <col min="2" max="2" customWidth="true" width="14.14"/>
-    <col min="3" max="3" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="27.29" customWidth="1"/>
+    <col min="2" max="2" width="14.14" customWidth="1"/>
+    <col min="3" max="3" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9344,14 +9296,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="29.43"/>
-    <col min="2" max="2" customWidth="true" width="31.43"/>
-    <col min="3" max="3" customWidth="true" width="28.71"/>
-    <col min="4" max="4" customWidth="true" width="30.57"/>
-    <col min="5" max="5" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="29.43" customWidth="1"/>
+    <col min="2" max="2" width="31.43" customWidth="1"/>
+    <col min="3" max="3" width="28.71" customWidth="1"/>
+    <col min="4" max="4" width="30.57" customWidth="1"/>
+    <col min="5" max="5" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9464,13 +9415,12 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.29"/>
-    <col min="2" max="2" customWidth="true" width="20.14"/>
-    <col min="3" max="4" customWidth="true" width="13.57"/>
-    <col min="5" max="5" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="27.29" customWidth="1"/>
+    <col min="2" max="2" width="20.14" customWidth="1"/>
+    <col min="3" max="4" width="13.57" customWidth="1"/>
+    <col min="5" max="5" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9569,12 +9519,11 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.57"/>
-    <col min="2" max="2" customWidth="true" width="39.86"/>
-    <col min="3" max="3" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="27.57" customWidth="1"/>
+    <col min="2" max="2" width="39.86" customWidth="1"/>
+    <col min="3" max="3" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9753,12 +9702,11 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="56.0"/>
-    <col min="2" max="2" customWidth="true" width="57.0"/>
-    <col min="3" max="3" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="56" customWidth="1"/>
+    <col min="2" max="2" width="57" customWidth="1"/>
+    <col min="3" max="3" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Updated the Selenium-java version - Numeric exception resolved.
</commit_message>
<xml_diff>
--- a/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
+++ b/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>TCID</t>
   </si>
@@ -340,12 +340,28 @@
   </si>
   <si>
     <t>Test Degree</t>
+  </si>
+  <si>
+    <t>Legal name</t>
+  </si>
+  <si>
+    <t>Test FN Automation MN Test LN</t>
+  </si>
+  <si>
+    <t>Preferred first name</t>
+  </si>
+  <si>
+    <t>Date of birth</t>
+  </si>
+  <si>
+    <t>November 23, 1933</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="9">
     <font>
       <sz val="11"/>
@@ -417,7 +433,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -440,6 +456,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -648,10 +673,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="24.57" customWidth="1"/>
-    <col min="2" max="6" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="24.57"/>
+    <col min="2" max="6" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2365,14 +2391,15 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="38.29" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="22.29" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="18.57" customWidth="1"/>
-    <col min="7" max="7" width="30.14" customWidth="1"/>
+    <col min="1" max="2" customWidth="true" width="38.29"/>
+    <col min="3" max="3" customWidth="true" width="34.0"/>
+    <col min="4" max="4" customWidth="true" width="22.29"/>
+    <col min="5" max="5" customWidth="true" width="30.0"/>
+    <col min="6" max="6" customWidth="true" width="18.57"/>
+    <col min="7" max="7" customWidth="true" width="30.14"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2464,13 +2491,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="38.29" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="22.29" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="14.43" customWidth="1"/>
+    <col min="1" max="2" customWidth="true" width="38.29"/>
+    <col min="3" max="3" customWidth="true" width="34.0"/>
+    <col min="4" max="4" customWidth="true" width="22.29"/>
+    <col min="5" max="5" customWidth="true" width="30.0"/>
+    <col min="6" max="6" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2544,13 +2572,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.14" customWidth="1"/>
-    <col min="2" max="2" width="29.57" customWidth="1"/>
-    <col min="3" max="3" width="41.43" customWidth="1"/>
-    <col min="4" max="4" width="34.43" customWidth="1"/>
-    <col min="5" max="5" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.14"/>
+    <col min="2" max="2" customWidth="true" width="29.57"/>
+    <col min="3" max="3" customWidth="true" width="41.43"/>
+    <col min="4" max="4" customWidth="true" width="34.43"/>
+    <col min="5" max="5" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2615,9 +2644,10 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="14.43" customWidth="1"/>
+    <col min="1" max="5" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2801,9 +2831,10 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="4" width="14.43" customWidth="1"/>
+    <col min="1" max="4" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2897,13 +2928,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31" customWidth="1"/>
-    <col min="2" max="2" width="27.43" customWidth="1"/>
-    <col min="3" max="3" width="51" customWidth="1"/>
-    <col min="4" max="4" width="22.43" customWidth="1"/>
-    <col min="5" max="5" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="31.0"/>
+    <col min="2" max="2" customWidth="true" width="27.43"/>
+    <col min="3" max="3" customWidth="true" width="51.0"/>
+    <col min="4" max="4" customWidth="true" width="22.43"/>
+    <col min="5" max="5" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2965,16 +2997,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="36.86" customWidth="1"/>
-    <col min="2" max="2" width="41.14" customWidth="1"/>
-    <col min="3" max="3" width="20.43" customWidth="1"/>
-    <col min="4" max="4" width="20.14" customWidth="1"/>
-    <col min="5" max="5" width="31.43" customWidth="1"/>
-    <col min="6" max="6" width="24.43" customWidth="1"/>
-    <col min="7" max="7" width="26.71" customWidth="1"/>
-    <col min="12" max="12" width="40.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="36.86"/>
+    <col min="2" max="2" customWidth="true" width="41.14"/>
+    <col min="3" max="3" customWidth="true" width="20.43"/>
+    <col min="4" max="4" customWidth="true" width="20.14"/>
+    <col min="5" max="5" customWidth="true" width="31.43"/>
+    <col min="6" max="6" customWidth="true" width="24.43"/>
+    <col min="7" max="7" customWidth="true" width="26.71"/>
+    <col min="12" max="12" customWidth="true" width="40.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -2988,8 +3021,12 @@
       <c r="L1" s="3"/>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="1"/>
-      <c r="B2" s="3"/>
+      <c r="A2" t="s" s="0">
+        <v>103</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>104</v>
+      </c>
       <c r="D2" s="3"/>
       <c r="E2" s="1"/>
       <c r="F2" s="3"/>
@@ -2998,8 +3035,12 @@
       <c r="L2" s="3"/>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" s="1"/>
-      <c r="B3" s="3"/>
+      <c r="A3" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>29</v>
+      </c>
       <c r="D3" s="3"/>
       <c r="E3" s="1"/>
       <c r="F3" s="3"/>
@@ -3008,8 +3049,12 @@
       <c r="L3" s="3"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" s="1"/>
-      <c r="B4" s="3"/>
+      <c r="A4" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>107</v>
+      </c>
       <c r="D4" s="3"/>
       <c r="E4" s="1"/>
       <c r="F4" s="3"/>
@@ -5108,14 +5153,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.14" customWidth="1"/>
-    <col min="2" max="2" width="23.71" customWidth="1"/>
-    <col min="3" max="3" width="45.14" customWidth="1"/>
-    <col min="4" max="4" width="14.57" customWidth="1"/>
-    <col min="5" max="5" width="60" customWidth="1"/>
-    <col min="6" max="6" width="25.14" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="13.14"/>
+    <col min="2" max="2" customWidth="true" width="23.71"/>
+    <col min="3" max="3" customWidth="true" width="45.14"/>
+    <col min="4" max="4" customWidth="true" width="14.57"/>
+    <col min="5" max="5" customWidth="true" width="60.0"/>
+    <col min="6" max="6" customWidth="true" width="25.14"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -7173,14 +7219,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="37.29" customWidth="1"/>
-    <col min="2" max="2" width="29.57" customWidth="1"/>
-    <col min="3" max="3" width="24.57" customWidth="1"/>
-    <col min="4" max="4" width="27.57" customWidth="1"/>
-    <col min="5" max="5" width="25.29" customWidth="1"/>
-    <col min="6" max="6" width="33.57" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="37.29"/>
+    <col min="2" max="2" customWidth="true" width="29.57"/>
+    <col min="3" max="3" customWidth="true" width="24.57"/>
+    <col min="4" max="4" customWidth="true" width="27.57"/>
+    <col min="5" max="5" customWidth="true" width="25.29"/>
+    <col min="6" max="6" customWidth="true" width="33.57"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9234,11 +9281,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.29" customWidth="1"/>
-    <col min="2" max="2" width="14.14" customWidth="1"/>
-    <col min="3" max="3" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.29"/>
+    <col min="2" max="2" customWidth="true" width="14.14"/>
+    <col min="3" max="3" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9296,13 +9344,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="29.43" customWidth="1"/>
-    <col min="2" max="2" width="31.43" customWidth="1"/>
-    <col min="3" max="3" width="28.71" customWidth="1"/>
-    <col min="4" max="4" width="30.57" customWidth="1"/>
-    <col min="5" max="5" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="29.43"/>
+    <col min="2" max="2" customWidth="true" width="31.43"/>
+    <col min="3" max="3" customWidth="true" width="28.71"/>
+    <col min="4" max="4" customWidth="true" width="30.57"/>
+    <col min="5" max="5" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9415,12 +9464,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.29" customWidth="1"/>
-    <col min="2" max="2" width="20.14" customWidth="1"/>
-    <col min="3" max="4" width="13.57" customWidth="1"/>
-    <col min="5" max="5" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.29"/>
+    <col min="2" max="2" customWidth="true" width="20.14"/>
+    <col min="3" max="4" customWidth="true" width="13.57"/>
+    <col min="5" max="5" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9519,11 +9569,12 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.57" customWidth="1"/>
-    <col min="2" max="2" width="39.86" customWidth="1"/>
-    <col min="3" max="3" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.57"/>
+    <col min="2" max="2" customWidth="true" width="39.86"/>
+    <col min="3" max="3" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9702,11 +9753,12 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="56" customWidth="1"/>
-    <col min="2" max="2" width="57" customWidth="1"/>
-    <col min="3" max="3" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="56.0"/>
+    <col min="2" max="2" customWidth="true" width="57.0"/>
+    <col min="3" max="3" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">

</xml_diff>

<commit_message>
My info updates till citizenship
</commit_message>
<xml_diff>
--- a/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
+++ b/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>TCID</t>
   </si>
@@ -340,19 +340,12 @@
   </si>
   <si>
     <t>Test Degree</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>2063622@test.asu.edu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="9">
     <font>
       <sz val="11"/>
@@ -424,7 +417,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -447,9 +440,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -658,11 +648,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="24.57"/>
-    <col min="2" max="6" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="24.57" customWidth="1"/>
+    <col min="2" max="6" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2376,15 +2365,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="38.29"/>
-    <col min="3" max="3" customWidth="true" width="34.0"/>
-    <col min="4" max="4" customWidth="true" width="22.29"/>
-    <col min="5" max="5" customWidth="true" width="30.0"/>
-    <col min="6" max="6" customWidth="true" width="18.57"/>
-    <col min="7" max="7" customWidth="true" width="30.14"/>
+    <col min="1" max="2" width="38.29" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="22.29" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="18.57" customWidth="1"/>
+    <col min="7" max="7" width="30.14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2476,14 +2464,13 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="38.29"/>
-    <col min="3" max="3" customWidth="true" width="34.0"/>
-    <col min="4" max="4" customWidth="true" width="22.29"/>
-    <col min="5" max="5" customWidth="true" width="30.0"/>
-    <col min="6" max="6" customWidth="true" width="14.43"/>
+    <col min="1" max="2" width="38.29" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="22.29" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2557,14 +2544,13 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.14"/>
-    <col min="2" max="2" customWidth="true" width="29.57"/>
-    <col min="3" max="3" customWidth="true" width="41.43"/>
-    <col min="4" max="4" customWidth="true" width="34.43"/>
-    <col min="5" max="5" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="27.14" customWidth="1"/>
+    <col min="2" max="2" width="29.57" customWidth="1"/>
+    <col min="3" max="3" width="41.43" customWidth="1"/>
+    <col min="4" max="4" width="34.43" customWidth="1"/>
+    <col min="5" max="5" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2629,10 +2615,9 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="5" customWidth="true" width="14.43"/>
+    <col min="1" max="5" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2816,10 +2801,9 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="4" customWidth="true" width="14.43"/>
+    <col min="1" max="4" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2913,14 +2897,13 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="31.0"/>
-    <col min="2" max="2" customWidth="true" width="27.43"/>
-    <col min="3" max="3" customWidth="true" width="51.0"/>
-    <col min="4" max="4" customWidth="true" width="22.43"/>
-    <col min="5" max="5" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="31" customWidth="1"/>
+    <col min="2" max="2" width="27.43" customWidth="1"/>
+    <col min="3" max="3" width="51" customWidth="1"/>
+    <col min="4" max="4" width="22.43" customWidth="1"/>
+    <col min="5" max="5" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2982,26 +2965,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="36.86"/>
-    <col min="2" max="2" customWidth="true" width="41.14"/>
-    <col min="3" max="3" customWidth="true" width="20.43"/>
-    <col min="4" max="4" customWidth="true" width="20.14"/>
-    <col min="5" max="5" customWidth="true" width="31.43"/>
-    <col min="6" max="6" customWidth="true" width="24.43"/>
-    <col min="7" max="7" customWidth="true" width="26.71"/>
-    <col min="12" max="12" customWidth="true" width="40.71"/>
+    <col min="1" max="1" width="36.86" customWidth="1"/>
+    <col min="2" max="2" width="41.14" customWidth="1"/>
+    <col min="3" max="3" width="20.43" customWidth="1"/>
+    <col min="4" max="4" width="20.14" customWidth="1"/>
+    <col min="5" max="5" width="31.43" customWidth="1"/>
+    <col min="6" max="6" width="24.43" customWidth="1"/>
+    <col min="7" max="7" width="26.71" customWidth="1"/>
+    <col min="12" max="12" width="40.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" t="s" s="0">
-        <v>103</v>
-      </c>
-      <c r="B1" s="14" t="s">
-        <v>104</v>
-      </c>
+      <c r="B1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="1"/>
       <c r="F1" s="3"/>
@@ -5131,15 +5108,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="13.14"/>
-    <col min="2" max="2" customWidth="true" width="23.71"/>
-    <col min="3" max="3" customWidth="true" width="45.14"/>
-    <col min="4" max="4" customWidth="true" width="14.57"/>
-    <col min="5" max="5" customWidth="true" width="60.0"/>
-    <col min="6" max="6" customWidth="true" width="25.14"/>
+    <col min="1" max="1" width="13.14" customWidth="1"/>
+    <col min="2" max="2" width="23.71" customWidth="1"/>
+    <col min="3" max="3" width="45.14" customWidth="1"/>
+    <col min="4" max="4" width="14.57" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
+    <col min="6" max="6" width="25.14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -7197,15 +7173,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="37.29"/>
-    <col min="2" max="2" customWidth="true" width="29.57"/>
-    <col min="3" max="3" customWidth="true" width="24.57"/>
-    <col min="4" max="4" customWidth="true" width="27.57"/>
-    <col min="5" max="5" customWidth="true" width="25.29"/>
-    <col min="6" max="6" customWidth="true" width="33.57"/>
+    <col min="1" max="1" width="37.29" customWidth="1"/>
+    <col min="2" max="2" width="29.57" customWidth="1"/>
+    <col min="3" max="3" width="24.57" customWidth="1"/>
+    <col min="4" max="4" width="27.57" customWidth="1"/>
+    <col min="5" max="5" width="25.29" customWidth="1"/>
+    <col min="6" max="6" width="33.57" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9259,12 +9234,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.29"/>
-    <col min="2" max="2" customWidth="true" width="14.14"/>
-    <col min="3" max="3" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="27.29" customWidth="1"/>
+    <col min="2" max="2" width="14.14" customWidth="1"/>
+    <col min="3" max="3" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9322,14 +9296,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="29.43"/>
-    <col min="2" max="2" customWidth="true" width="31.43"/>
-    <col min="3" max="3" customWidth="true" width="28.71"/>
-    <col min="4" max="4" customWidth="true" width="30.57"/>
-    <col min="5" max="5" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="29.43" customWidth="1"/>
+    <col min="2" max="2" width="31.43" customWidth="1"/>
+    <col min="3" max="3" width="28.71" customWidth="1"/>
+    <col min="4" max="4" width="30.57" customWidth="1"/>
+    <col min="5" max="5" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9442,13 +9415,12 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.29"/>
-    <col min="2" max="2" customWidth="true" width="20.14"/>
-    <col min="3" max="4" customWidth="true" width="13.57"/>
-    <col min="5" max="5" customWidth="true" width="8.71"/>
+    <col min="1" max="1" width="27.29" customWidth="1"/>
+    <col min="2" max="2" width="20.14" customWidth="1"/>
+    <col min="3" max="4" width="13.57" customWidth="1"/>
+    <col min="5" max="5" width="8.71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9547,12 +9519,11 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.57"/>
-    <col min="2" max="2" customWidth="true" width="39.86"/>
-    <col min="3" max="3" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="27.57" customWidth="1"/>
+    <col min="2" max="2" width="39.86" customWidth="1"/>
+    <col min="3" max="3" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9731,12 +9702,11 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="56.0"/>
-    <col min="2" max="2" customWidth="true" width="57.0"/>
-    <col min="3" max="3" customWidth="true" width="14.43"/>
+    <col min="1" max="1" width="56" customWidth="1"/>
+    <col min="2" max="2" width="57" customWidth="1"/>
+    <col min="3" max="3" width="14.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Latest code - Includes a review of the folder structures, followed by a refactor.
</commit_message>
<xml_diff>
--- a/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
+++ b/UAA/src/src/test/resources/com/ugapp/excel/testdata.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>TCID</t>
   </si>
@@ -340,12 +340,19 @@
   </si>
   <si>
     <t>Test Degree</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>7104246@test.asu.edu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="9">
     <font>
       <sz val="11"/>
@@ -417,7 +424,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -440,6 +447,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -648,10 +658,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="24.57" customWidth="1"/>
-    <col min="2" max="6" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="24.57"/>
+    <col min="2" max="6" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2365,14 +2376,15 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="38.29" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="22.29" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="18.57" customWidth="1"/>
-    <col min="7" max="7" width="30.14" customWidth="1"/>
+    <col min="1" max="2" customWidth="true" width="38.29"/>
+    <col min="3" max="3" customWidth="true" width="34.0"/>
+    <col min="4" max="4" customWidth="true" width="22.29"/>
+    <col min="5" max="5" customWidth="true" width="30.0"/>
+    <col min="6" max="6" customWidth="true" width="18.57"/>
+    <col min="7" max="7" customWidth="true" width="30.14"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2464,13 +2476,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="38.29" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="22.29" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="14.43" customWidth="1"/>
+    <col min="1" max="2" customWidth="true" width="38.29"/>
+    <col min="3" max="3" customWidth="true" width="34.0"/>
+    <col min="4" max="4" customWidth="true" width="22.29"/>
+    <col min="5" max="5" customWidth="true" width="30.0"/>
+    <col min="6" max="6" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2544,13 +2557,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.14" customWidth="1"/>
-    <col min="2" max="2" width="29.57" customWidth="1"/>
-    <col min="3" max="3" width="41.43" customWidth="1"/>
-    <col min="4" max="4" width="34.43" customWidth="1"/>
-    <col min="5" max="5" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.14"/>
+    <col min="2" max="2" customWidth="true" width="29.57"/>
+    <col min="3" max="3" customWidth="true" width="41.43"/>
+    <col min="4" max="4" customWidth="true" width="34.43"/>
+    <col min="5" max="5" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2615,9 +2629,10 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="14.43" customWidth="1"/>
+    <col min="1" max="5" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2801,9 +2816,10 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="4" width="14.43" customWidth="1"/>
+    <col min="1" max="4" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2897,13 +2913,14 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31" customWidth="1"/>
-    <col min="2" max="2" width="27.43" customWidth="1"/>
-    <col min="3" max="3" width="51" customWidth="1"/>
-    <col min="4" max="4" width="22.43" customWidth="1"/>
-    <col min="5" max="5" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="31.0"/>
+    <col min="2" max="2" customWidth="true" width="27.43"/>
+    <col min="3" max="3" customWidth="true" width="51.0"/>
+    <col min="4" max="4" customWidth="true" width="22.43"/>
+    <col min="5" max="5" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -2965,20 +2982,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="36.86" customWidth="1"/>
-    <col min="2" max="2" width="41.14" customWidth="1"/>
-    <col min="3" max="3" width="20.43" customWidth="1"/>
-    <col min="4" max="4" width="20.14" customWidth="1"/>
-    <col min="5" max="5" width="31.43" customWidth="1"/>
-    <col min="6" max="6" width="24.43" customWidth="1"/>
-    <col min="7" max="7" width="26.71" customWidth="1"/>
-    <col min="12" max="12" width="40.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="36.86"/>
+    <col min="2" max="2" customWidth="true" width="41.14"/>
+    <col min="3" max="3" customWidth="true" width="20.43"/>
+    <col min="4" max="4" customWidth="true" width="20.14"/>
+    <col min="5" max="5" customWidth="true" width="31.43"/>
+    <col min="6" max="6" customWidth="true" width="24.43"/>
+    <col min="7" max="7" customWidth="true" width="26.71"/>
+    <col min="12" max="12" customWidth="true" width="40.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="B1" s="3"/>
+      <c r="A1" t="s" s="0">
+        <v>103</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>104</v>
+      </c>
       <c r="D1" s="3"/>
       <c r="E1" s="1"/>
       <c r="F1" s="3"/>
@@ -5108,14 +5131,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.14" customWidth="1"/>
-    <col min="2" max="2" width="23.71" customWidth="1"/>
-    <col min="3" max="3" width="45.14" customWidth="1"/>
-    <col min="4" max="4" width="14.57" customWidth="1"/>
-    <col min="5" max="5" width="60" customWidth="1"/>
-    <col min="6" max="6" width="25.14" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="13.14"/>
+    <col min="2" max="2" customWidth="true" width="23.71"/>
+    <col min="3" max="3" customWidth="true" width="45.14"/>
+    <col min="4" max="4" customWidth="true" width="14.57"/>
+    <col min="5" max="5" customWidth="true" width="60.0"/>
+    <col min="6" max="6" customWidth="true" width="25.14"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -7173,14 +7197,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="37.29" customWidth="1"/>
-    <col min="2" max="2" width="29.57" customWidth="1"/>
-    <col min="3" max="3" width="24.57" customWidth="1"/>
-    <col min="4" max="4" width="27.57" customWidth="1"/>
-    <col min="5" max="5" width="25.29" customWidth="1"/>
-    <col min="6" max="6" width="33.57" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="37.29"/>
+    <col min="2" max="2" customWidth="true" width="29.57"/>
+    <col min="3" max="3" customWidth="true" width="24.57"/>
+    <col min="4" max="4" customWidth="true" width="27.57"/>
+    <col min="5" max="5" customWidth="true" width="25.29"/>
+    <col min="6" max="6" customWidth="true" width="33.57"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9234,11 +9259,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.29" customWidth="1"/>
-    <col min="2" max="2" width="14.14" customWidth="1"/>
-    <col min="3" max="3" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.29"/>
+    <col min="2" max="2" customWidth="true" width="14.14"/>
+    <col min="3" max="3" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9296,13 +9322,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="29.43" customWidth="1"/>
-    <col min="2" max="2" width="31.43" customWidth="1"/>
-    <col min="3" max="3" width="28.71" customWidth="1"/>
-    <col min="4" max="4" width="30.57" customWidth="1"/>
-    <col min="5" max="5" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="29.43"/>
+    <col min="2" max="2" customWidth="true" width="31.43"/>
+    <col min="3" max="3" customWidth="true" width="28.71"/>
+    <col min="4" max="4" customWidth="true" width="30.57"/>
+    <col min="5" max="5" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -9415,12 +9442,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.29" customWidth="1"/>
-    <col min="2" max="2" width="20.14" customWidth="1"/>
-    <col min="3" max="4" width="13.57" customWidth="1"/>
-    <col min="5" max="5" width="8.71" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.29"/>
+    <col min="2" max="2" customWidth="true" width="20.14"/>
+    <col min="3" max="4" customWidth="true" width="13.57"/>
+    <col min="5" max="5" customWidth="true" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9519,11 +9547,12 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.57" customWidth="1"/>
-    <col min="2" max="2" width="39.86" customWidth="1"/>
-    <col min="3" max="3" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.57"/>
+    <col min="2" max="2" customWidth="true" width="39.86"/>
+    <col min="3" max="3" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -9702,11 +9731,12 @@
   <sheetPr>
     <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="56" customWidth="1"/>
-    <col min="2" max="2" width="57" customWidth="1"/>
-    <col min="3" max="3" width="14.43" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="56.0"/>
+    <col min="2" max="2" customWidth="true" width="57.0"/>
+    <col min="3" max="3" customWidth="true" width="14.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">

</xml_diff>